<commit_message>
chore(config): add New-AccountsTemplate.ps1 and regenerate Accounts.template.xlsx, refs #57
New-AccountsTemplate.ps1 generates Config/Accounts.template.xlsx using
Excel COM. Reads method tokens from Config/Methods.template.json and
prepends Cash. New schema: Last 4, Method, Holder, Institution, Account,
Status with dropdown validation on Method (blank allowed) and Status
(required stop alert). Run whenever the Accounts schema changes.
</commit_message>
<xml_diff>
--- a/Config/Accounts.template.xlsx
+++ b/Config/Accounts.template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="f:\Documents\Sync-Receipts\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://peplinskigroup-my.sharepoint.com/personal/ndomako_peplinskigroup_com/Documents/Workspace/Repos/Sync-Receipts/Config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{23AED375-DA43-4F13-A5CD-AB99667C0C9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{72F9114D-47DC-4361-8827-0F9EFD8D35A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CBA46100-9164-42DE-B79D-BCBCEC8B08F6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D7436DFD-F471-486A-BF24-2F4E613CA9E8}"/>
   </bookViews>
   <sheets>
     <sheet name="Accounts" sheetId="1" r:id="rId1"/>
@@ -36,69 +36,45 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="13">
   <si>
     <t>Last 4</t>
   </si>
   <si>
+    <t>Method</t>
+  </si>
+  <si>
     <t>Holder</t>
   </si>
   <si>
     <t>Institution</t>
   </si>
   <si>
-    <t>Network</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>1234</t>
-  </si>
-  <si>
-    <t>John Doe</t>
-  </si>
-  <si>
-    <t>Example Bank</t>
-  </si>
-  <si>
-    <t>Visa</t>
-  </si>
-  <si>
-    <t>Credit</t>
-  </si>
-  <si>
-    <t>5678</t>
-  </si>
-  <si>
-    <t>Mastercard</t>
-  </si>
-  <si>
-    <t>Debit</t>
-  </si>
-  <si>
-    <t>6310</t>
+    <t>Account</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Card</t>
+  </si>
+  <si>
+    <t>Account Holder</t>
+  </si>
+  <si>
+    <t>Institution Name</t>
+  </si>
+  <si>
+    <t>Checking Account Name</t>
+  </si>
+  <si>
+    <t>Active</t>
   </si>
   <si>
     <t>Checking</t>
   </si>
   <si>
-    <t>Savings</t>
-  </si>
-  <si>
-    <t>0943</t>
-  </si>
-  <si>
-    <t>Jane Doe</t>
-  </si>
-  <si>
-    <t>EBT</t>
-  </si>
-  <si>
-    <t>0000</t>
-  </si>
-  <si>
-    <t>Cash</t>
+    <t>Check</t>
   </si>
 </sst>
 </file>
@@ -134,18 +110,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
-    <dxf>
-      <numFmt numFmtId="30" formatCode="@"/>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -159,14 +130,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{50309A1C-B440-4A59-8CE6-73E87C578C87}" name="Accounts" displayName="Accounts" ref="A1:E7" totalsRowShown="0">
-  <autoFilter ref="A1:E7" xr:uid="{50309A1C-B440-4A59-8CE6-73E87C578C87}"/>
-  <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{1EB8C79E-FC90-465D-8868-1F043F162229}" name="Last 4" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{96F63431-C3B1-47B4-9374-945E3C9B425A}" name="Holder"/>
-    <tableColumn id="3" xr3:uid="{3F67CA97-4731-479F-8F5B-1D974FC709D1}" name="Institution"/>
-    <tableColumn id="4" xr3:uid="{09C18D87-349A-4EDD-90CE-A7C5A4B115A0}" name="Network"/>
-    <tableColumn id="5" xr3:uid="{844ADA0F-183E-4348-87B7-4052A77188E2}" name="Type"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{78FCB28D-D0B8-43D6-A774-9DCDFC60D9C5}" name="Accounts" displayName="Accounts" ref="A1:F5" totalsRowShown="0">
+  <autoFilter ref="A1:F5" xr:uid="{78FCB28D-D0B8-43D6-A774-9DCDFC60D9C5}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{B5CFEB88-FF35-4775-92EA-EAE09A9CAF80}" name="Last 4"/>
+    <tableColumn id="2" xr3:uid="{D98CF599-A1D2-4899-A974-63016089911F}" name="Method"/>
+    <tableColumn id="3" xr3:uid="{11047B9C-1757-433C-9B9C-D60C416D7E35}" name="Holder"/>
+    <tableColumn id="4" xr3:uid="{606A5EA9-0F60-4103-A124-93539CAC744F}" name="Institution"/>
+    <tableColumn id="5" xr3:uid="{F3474CB6-049C-4055-B57A-3EFD906905DC}" name="Account"/>
+    <tableColumn id="6" xr3:uid="{243DC093-932C-4C60-966A-8D24C01541C2}" name="Status"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -488,19 +460,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CCB5D12-F6A7-47F5-92E8-B7EC76E1230A}">
-  <dimension ref="A1:E7"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51C5B45E-E739-4DD4-AE4E-542775DD5CAD}">
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.7109375" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" customWidth="1"/>
+    <col min="3" max="4" width="20.7109375" customWidth="1"/>
+    <col min="5" max="5" width="25.7109375" customWidth="1"/>
+    <col min="6" max="6" width="12.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
@@ -515,10 +487,13 @@
       <c r="E1" t="s">
         <v>4</v>
       </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>5</v>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1234</v>
       </c>
       <c r="B2" t="s">
         <v>6</v>
@@ -532,78 +507,76 @@
       <c r="E2" t="s">
         <v>9</v>
       </c>
+      <c r="F2" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>6</v>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>5678</v>
       </c>
       <c r="C3" t="s">
         <v>7</v>
       </c>
       <c r="D3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>9012</v>
+      </c>
+      <c r="B4" t="s">
         <v>11</v>
-      </c>
-      <c r="E3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" t="s">
-        <v>6</v>
       </c>
       <c r="C4" t="s">
         <v>7</v>
       </c>
+      <c r="D4" t="s">
+        <v>8</v>
+      </c>
       <c r="E4" t="s">
-        <v>14</v>
+        <v>9</v>
+      </c>
+      <c r="F4" t="s">
+        <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>13</v>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>9012</v>
       </c>
       <c r="B5" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="C5" t="s">
         <v>7</v>
       </c>
+      <c r="D5" t="s">
+        <v>8</v>
+      </c>
       <c r="E5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" t="s">
-        <v>18</v>
-      </c>
-      <c r="E6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" t="s">
-        <v>6</v>
-      </c>
-      <c r="E7" t="s">
-        <v>20</v>
+        <v>9</v>
+      </c>
+      <c r="F5" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="list" errorStyle="information" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B1048576" xr:uid="{447155E5-2EB4-4A4A-A154-E4063C785BA1}">
+      <formula1>"Cash,Card,Check,Checking,Savings,Transfer,Wire"</formula1>
+    </dataValidation>
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="F2:F1048576" xr:uid="{385DBACC-3158-483F-9561-22F5F2F829B4}">
+      <formula1>"Active,Inactive"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>